<commit_message>
fix: correct TRK_DN directionality to NOMINAL and align Down line signals (RHS-CORRECTION-COMPREHENSIVE-DIR-001)
- Set TRK_DN DIRECTIONALITY to NOMINAL in generate.py and regenerated workbooks, aligning permitted traversal with South-to-North link orientations (ND_11 to ND_01).
- Updated SIG_DN_01..07 direction to NOMINAL to govern forward traversal along Down line track links.
- Updated examples/05_comprehensive_line/README.md to document NOMINAL track directionality semantics and Down line routes.
- Added regression tests verifying declared directionality matches permitted routes for all tracks and guarding against directionality reversals.
- Confirmed AN_HSR_HSR_DN and AN_REG_REG_DN resolve successfully.
- Updated DEVELOPMENT_MANIFEST.md with 777 passing tests.
</commit_message>
<xml_diff>
--- a/examples/05_comprehensive_line/02_Signalling.xlsx
+++ b/examples/05_comprehensive_line/02_Signalling.xlsx
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>REVERSE</t>
+          <t>NOMINAL</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">

</xml_diff>